<commit_message>
feat: foglio Simulazione_M2 - madre muore a M2, C2 diventa madre e copre speso+target
</commit_message>
<xml_diff>
--- a/Modello_Multiplatore_a_Scalare.xlsx
+++ b/Modello_Multiplatore_a_Scalare.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assicurazione" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutte_Situazioni" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formule" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simulazione_M2" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4282,4 +4283,574 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SIMULAZIONE - Madre muore alla 2a partita (15 eventi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>M1 Under (Madre attiva), M2 OVER (Madre muore, 2EUR persi), C2 diventa madre: la sua vincita copre speso precedente + target</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Evento</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Esito</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Ticket Attivo</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>N_pending</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Finale</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Stake</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Spesa_cum</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Lordo</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Netto</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>S0/M1</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Under</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Madre</t>
+        </is>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="F5" s="9">
+        <f>1.32^15</f>
+        <v/>
+      </c>
+      <c r="G5" s="9">
+        <f>F5*(1+89.8/100)</f>
+        <v/>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" s="8">
+        <f>H5*G5</f>
+        <v/>
+      </c>
+      <c r="K5" s="8">
+        <f>J5-I5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>OVER</t>
+        </is>
+      </c>
+      <c r="D6" s="23" t="inlineStr">
+        <is>
+          <t>S0-&gt;C2</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="n">
+        <v>13</v>
+      </c>
+      <c r="F6" s="25">
+        <f>1.32^13</f>
+        <v/>
+      </c>
+      <c r="G6" s="25">
+        <f>F6*(1+68.9/100)</f>
+        <v/>
+      </c>
+      <c r="H6" s="23">
+        <f>ROUNDUP((I5+45)/(G6-1)/0.5,0)*0.5</f>
+        <v/>
+      </c>
+      <c r="I6" s="23">
+        <f>I5+H6</f>
+        <v/>
+      </c>
+      <c r="J6" s="23">
+        <f>H6*G6</f>
+        <v/>
+      </c>
+      <c r="K6" s="23">
+        <f>J6-I6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>C2/M3</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Under</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>C2 (=madre)</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="F7" s="11">
+        <f>1.32^12</f>
+        <v/>
+      </c>
+      <c r="G7" s="11">
+        <f>F7*(1+59.4/100)</f>
+        <v/>
+      </c>
+      <c r="H7" s="6">
+        <f>ROUNDUP((I6+45)/(G7-1)/0.5,0)*0.5</f>
+        <v/>
+      </c>
+      <c r="I7" s="6">
+        <f>I6+H7</f>
+        <v/>
+      </c>
+      <c r="J7" s="6">
+        <f>H7*G7</f>
+        <v/>
+      </c>
+      <c r="K7" s="6">
+        <f>J7-I7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>C2/M4</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Under</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>C2 (=madre)</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="F8" s="11">
+        <f>1.32^11</f>
+        <v/>
+      </c>
+      <c r="G8" s="11">
+        <f>F8*(1+50.4/100)</f>
+        <v/>
+      </c>
+      <c r="H8" s="6">
+        <f>ROUNDUP((I7+45)/(G8-1)/0.5,0)*0.5</f>
+        <v/>
+      </c>
+      <c r="I8" s="6">
+        <f>I7+H8</f>
+        <v/>
+      </c>
+      <c r="J8" s="6">
+        <f>H8*G8</f>
+        <v/>
+      </c>
+      <c r="K8" s="6">
+        <f>J8-I8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>C2/M5</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Under</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>C2 (=madre)</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" s="11">
+        <f>1.32^10</f>
+        <v/>
+      </c>
+      <c r="G9" s="11">
+        <f>F9*(1+41.9/100)</f>
+        <v/>
+      </c>
+      <c r="H9" s="6">
+        <f>ROUNDUP((I8+45)/(G9-1)/0.5,0)*0.5</f>
+        <v/>
+      </c>
+      <c r="I9" s="6">
+        <f>I8+H9</f>
+        <v/>
+      </c>
+      <c r="J9" s="6">
+        <f>H9*G9</f>
+        <v/>
+      </c>
+      <c r="K9" s="6">
+        <f>J9-I9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>C2/M6</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Under</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>C2 (=madre)</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="F10" s="11">
+        <f>1.32^9</f>
+        <v/>
+      </c>
+      <c r="G10" s="11">
+        <f>F10*(1+33.8/100)</f>
+        <v/>
+      </c>
+      <c r="H10" s="6">
+        <f>ROUNDUP((I9+45)/(G10-1)/0.5,0)*0.5</f>
+        <v/>
+      </c>
+      <c r="I10" s="6">
+        <f>I9+H10</f>
+        <v/>
+      </c>
+      <c r="J10" s="6">
+        <f>H10*G10</f>
+        <v/>
+      </c>
+      <c r="K10" s="6">
+        <f>J10-I10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>C2/M7</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Under</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>C2 (=madre)</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="F11" s="11">
+        <f>1.32^8</f>
+        <v/>
+      </c>
+      <c r="G11" s="11">
+        <f>F11*(1+26.2/100)</f>
+        <v/>
+      </c>
+      <c r="H11" s="6">
+        <f>ROUNDUP((I10+45)/(G11-1)/0.5,0)*0.5</f>
+        <v/>
+      </c>
+      <c r="I11" s="6">
+        <f>I10+H11</f>
+        <v/>
+      </c>
+      <c r="J11" s="6">
+        <f>H11*G11</f>
+        <v/>
+      </c>
+      <c r="K11" s="6">
+        <f>J11-I11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Lock</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Exchange</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>LOCK</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Exchange</t>
+        </is>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="H12" s="8">
+        <f>ROUNDUP((I11+45)/(G12-1)/0.5,0)*0.5</f>
+        <v/>
+      </c>
+      <c r="I12" s="8">
+        <f>I11+H12</f>
+        <v/>
+      </c>
+      <c r="J12" s="8">
+        <f>H12*G12</f>
+        <v/>
+      </c>
+      <c r="K12" s="8">
+        <f>J12-I12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>VERIFICA ROLLOVER</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Perso con S0 (M2 Over)</t>
+        </is>
+      </c>
+      <c r="B15" s="6">
+        <f>I5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Stake C2 piazzata</t>
+        </is>
+      </c>
+      <c r="B16" s="6">
+        <f>H6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Spesa totale se C2 vince subito</t>
+        </is>
+      </c>
+      <c r="B17" s="5">
+        <f>I6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Lordo C2 (copre speso + target?)</t>
+        </is>
+      </c>
+      <c r="B18" s="13">
+        <f>J6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Netto C2 (&gt;=45 = rollover OK)</t>
+        </is>
+      </c>
+      <c r="B19" s="13">
+        <f>K6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Costo totale ciclo (fino a lock)</t>
+        </is>
+      </c>
+      <c r="B20" s="5">
+        <f>I12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Netto Lock</t>
+        </is>
+      </c>
+      <c r="B21" s="6">
+        <f>K12</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>